<commit_message>
feat : methode say hello
</commit_message>
<xml_diff>
--- a/data/yassine el  jabri.xlsx
+++ b/data/yassine el  jabri.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
   <si>
     <t xml:space="preserve">TEL CLIENT</t>
   </si>
@@ -37,6 +37,9 @@
     <t xml:space="preserve">+212661250473</t>
   </si>
   <si>
+    <t xml:space="preserve">18924.38a</t>
+  </si>
+  <si>
     <t xml:space="preserve">+212611250473</t>
   </si>
   <si>
@@ -47,6 +50,9 @@
   </si>
   <si>
     <t xml:space="preserve">+212611111111</t>
+  </si>
+  <si>
+    <t xml:space="preserve">999.12s</t>
   </si>
 </sst>
 </file>
@@ -194,8 +200,8 @@
       <c r="B3" s="2" t="n">
         <v>3174265</v>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>18924.38</v>
+      <c r="C3" s="2" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -211,7 +217,7 @@
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>123</v>
@@ -222,7 +228,7 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>234</v>
@@ -233,7 +239,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>234</v>
@@ -244,13 +250,13 @@
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>999</v>
       </c>
-      <c r="C8" s="2" t="n">
-        <v>999</v>
+      <c r="C8" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>